<commit_message>
Update USEI01 and USEI05 documentation
</commit_message>
<xml_diff>
--- a/sql-scripts/Dataset_Sprint_1_ com inserts.xlsx
+++ b/sql-scripts/Dataset_Sprint_1_ com inserts.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\IdeaProjects\sem-pi-25-26-g054\sql-scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diogo\IdeaProjects\sem3-pi-25-26-g054-repo\sql-scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62CCE598-4132-4730-B8CA-5A79B652FF21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{593F0165-5543-48D3-B6FF-C980A17B48A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="1" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Facility" sheetId="1" r:id="rId1"/>
@@ -1768,73 +1768,73 @@
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B18" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A3&amp;","&amp;E3&amp;","&amp;F3&amp;",1,"&amp;C3&amp;",1,"&amp;B3&amp;");"</f>
+        <f t="shared" ref="B18:B29" si="0">"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A3&amp;","&amp;E3&amp;","&amp;F3&amp;",1,"&amp;C3&amp;",1,"&amp;B3&amp;");"</f>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (10,8000,29003,1,1,1,2);</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B19" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A4&amp;","&amp;E4&amp;","&amp;F4&amp;",1,"&amp;C4&amp;",1,"&amp;B4&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (11,8000,10000,1,2,1,2);</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B20" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A5&amp;","&amp;E5&amp;","&amp;F5&amp;",1,"&amp;C5&amp;",1,"&amp;B5&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (15,8000,5286,1,1,1,3);</v>
       </c>
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B21" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A6&amp;","&amp;E6&amp;","&amp;F6&amp;",1,"&amp;C6&amp;",1,"&amp;B6&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (16,8000,6000,1,2,1,3);</v>
       </c>
     </row>
     <row r="22" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B22" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A7&amp;","&amp;E7&amp;","&amp;F7&amp;",1,"&amp;C7&amp;",1,"&amp;B7&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (14,8000,10387,1,1,1,4);</v>
       </c>
     </row>
     <row r="23" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B23" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A8&amp;","&amp;E8&amp;","&amp;F8&amp;",1,"&amp;C8&amp;",1,"&amp;B8&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (12,8000,12000,1,2,1,4);</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B24" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A9&amp;","&amp;E9&amp;","&amp;F9&amp;",1,"&amp;C9&amp;",1,"&amp;B9&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (13,6400,8000,1,3,1,4);</v>
       </c>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B25" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A10&amp;","&amp;E10&amp;","&amp;F10&amp;",1,"&amp;C10&amp;",1,"&amp;B10&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (20,8000,6000,1,1,1,5);</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B26" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A11&amp;","&amp;E11&amp;","&amp;F11&amp;",1,"&amp;C11&amp;",1,"&amp;B11&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (21,8000,3000,1,2,1,5);</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B27" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A12&amp;","&amp;E12&amp;","&amp;F12&amp;",1,"&amp;C12&amp;",1,"&amp;B12&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (22,8000,15000,1,3,1,5);</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B28" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A13&amp;","&amp;E13&amp;","&amp;F13&amp;",1,"&amp;C13&amp;",1,"&amp;B13&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (25,8000,20829,1,1,1,6);</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B29" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES ("&amp;A14&amp;","&amp;E14&amp;","&amp;F14&amp;",1,"&amp;C14&amp;",1,"&amp;B14&amp;");"</f>
+        <f t="shared" si="0"/>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmantesOrder,lineSegmentsTypeid, lineId) VALUES (26,8000,4264,1,1,1,7);</v>
       </c>
     </row>

</xml_diff>

<commit_message>
USBD21 relational model update USBD21 create tables and inserts
</commit_message>
<xml_diff>
--- a/sql-scripts/Dataset_Sprint_1_ com inserts.xlsx
+++ b/sql-scripts/Dataset_Sprint_1_ com inserts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diogo\IdeaProjects\sem3-pi-25-26-g054-repo\sql-scripts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\IdeaProjects\sem-pi-25-26-g054\sql-scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{593F0165-5543-48D3-B6FF-C980A17B48A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A490D747-0529-4741-9567-08B759357A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" activeTab="5" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Facility" sheetId="1" r:id="rId1"/>
@@ -487,13 +487,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2220,7 +2221,7 @@
       <c r="I5" t="s">
         <v>118</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="6" t="s">
         <v>119</v>
       </c>
       <c r="K5" t="s">

</xml_diff>